<commit_message>
tracking update 16.07.2026 01:01
</commit_message>
<xml_diff>
--- a/files/UAE-003_ФПЗ_10.06.2026.xlsx
+++ b/files/UAE-003_ФПЗ_10.06.2026.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zinov\OneDrive\Desktop\РАБОЧАЯ\001 ИМПОРТ\001 containers\2026\001 UAE\UAE#3_DO_NOT_COUNT\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zinov\OneDrive\Desktop\РАБОЧАЯ\001 ИМПОРТ\001 containers\2026\001 UAE\UAE#3_APMG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{612B51C1-5B71-4187-AD4C-37567521AF6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DCAAE9B-B1C7-490A-A80E-703A3C33E493}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1545" yWindow="1830" windowWidth="35295" windowHeight="18060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1905" yWindow="1905" windowWidth="35295" windowHeight="18060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ФПЗ_Э3" sheetId="1" r:id="rId1"/>
@@ -4109,7 +4109,7 @@
         <v>933.63695510735215</v>
       </c>
       <c r="S4" s="29">
-        <f t="shared" ref="S3:S4" si="6">O4+P4+Q4+R4</f>
+        <f t="shared" ref="S4" si="6">O4+P4+Q4+R4</f>
         <v>634773.74710908695</v>
       </c>
       <c r="T4" s="30">

</xml_diff>